<commit_message>
Added url column in test data excel
</commit_message>
<xml_diff>
--- a/src/test/resources/test_data_template.xlsx
+++ b/src/test/resources/test_data_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rugvedgundawar/Documents/Group2-selenium-automation-project/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sarthak\sqcm\Group2-selenium-automation-project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BF3AC0-45D7-CD4A-92FA-97CD97AF4970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFA2FE7-8820-48FC-8D9B-2D8A6CC844E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t>username</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>username@northeastern.edu</t>
+  </si>
+  <si>
+    <t>url</t>
   </si>
 </sst>
 </file>
@@ -549,22 +552,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>38</v>
       </c>
@@ -583,7 +590,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -592,7 +599,7 @@
     <col min="6" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -612,7 +619,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>35</v>
       </c>
@@ -632,7 +639,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>36</v>
       </c>
@@ -660,17 +667,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -683,14 +690,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -701,7 +708,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
@@ -712,7 +719,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -723,7 +730,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -734,7 +741,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -745,7 +752,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -756,7 +763,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -767,7 +774,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -778,7 +785,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -789,7 +796,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>

</xml_diff>